<commit_message>
Ejecuto bloque Home y registro resultados en matriz
</commit_message>
<xml_diff>
--- a/casos_de_prueba/matriz_pruebas.xlsx
+++ b/casos_de_prueba/matriz_pruebas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USUARIO\Desktop\ProyectoFinal-QA-Scarleth\casos_de_prueba\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C626E798-76C5-4274-8D18-F0FFB5F300AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73F084C9-E377-426F-8528-781A64ABABC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{5FF4DDCA-2057-4105-B76A-F7B3AA90F74B}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="66">
   <si>
     <t>ID</t>
   </si>
@@ -60,15 +60,213 @@
   </si>
   <si>
     <t>Severidad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Categoria </t>
+  </si>
+  <si>
+    <t>CP01</t>
+  </si>
+  <si>
+    <t>Home/feed</t>
+  </si>
+  <si>
+    <t>1. Abrir chrome 2.Abrir pinterst. 3. Observar que sucede en los primeros segundos de la pagina.</t>
+  </si>
+  <si>
+    <t>La pagina carga sin problemas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tras que se ve la pagina lanza estructura intuitiva y sugerencias de interes. </t>
+  </si>
+  <si>
+    <t>Alta</t>
+  </si>
+  <si>
+    <t>Baja</t>
+  </si>
+  <si>
+    <t>Estado</t>
+  </si>
+  <si>
+    <t>OK</t>
+  </si>
+  <si>
+    <t>CP02</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Siempre en el home de pinterest. 1. Ir a la esquina superior izquierda a la parte de "explorar". 2. Visualizar al menos 10 imagenes de forma secuencial.</t>
+  </si>
+  <si>
+    <t>Conexion estable.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El home muestra secuencia de imagenes fluidas. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Navegar en angulo de al menos 10 imagenes. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">La pagina permite ver diferentes imagenes. </t>
+  </si>
+  <si>
+    <t>Media</t>
+  </si>
+  <si>
+    <t>Las imágenes cargan correctamente. En la última fila quedan espacios vacíos sin mensaje, pero no afecta funcionalidad ni navegación.</t>
+  </si>
+  <si>
+    <t>CP03</t>
+  </si>
+  <si>
+    <t>Verificar comportamiento dinámico de carga.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hacer scroll continuo hasta que el sistema no cargue mas. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Siempre en la parte de explorar. 1. Subir y bajar continuamente. 2. Bajar la home hasta que no cargue mas. </t>
+  </si>
+  <si>
+    <t>El sistema permite scroll hasta cierto límite y luego restringe contenido sin generar errores.</t>
+  </si>
+  <si>
+    <t>Se permite scroll hasta X cantidad de imágenes. Luego deja de cargar más contenido sin bloquear la navegación.</t>
+  </si>
+  <si>
+    <t>Observaciones</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Al llegar al limite del home no tira mensaje de logearse para ver mas. </t>
+  </si>
+  <si>
+    <t>CP04</t>
+  </si>
+  <si>
+    <t>Validar que al refrescar la página no se rompa el feed y vuelva a cargar correctamente.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recargar la pagina estando en la parte final de la misma (donde da el limit). </t>
+  </si>
+  <si>
+    <t xml:space="preserve">En la parte final la pagina (cuando da el limite). 1. Presionar F5.  2. Esperar a que cargue. 3. Observar la respuesta que dio el refresh. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">La pagina carga nuevamente sin salirse de donde se hizo el refresh. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">La pagina no se sale desde donde se hizo el refresh y volvio al inicio de la misma, mostrando las mismas imagenes anteriores. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validar que el home de la pagina responde rapido. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">CP05 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validar la respuesta de los pines. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seleccionar 1 pin para ver la respuesta. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Tocar un pin de la feed que nos muestra. 2. Observar que aparece al clickear el pin.  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">El pin abre correctamente, mostrando la imagen seleccionada y relacionados. </t>
+  </si>
+  <si>
+    <t>La imagen abrio correctamente y surgirio relacionados.</t>
+  </si>
+  <si>
+    <t>CP06</t>
+  </si>
+  <si>
+    <t>Verificar el resultado del "regresar".</t>
+  </si>
+  <si>
+    <t>1. Con el pin abierto, presiona el botón Atrás del navegador.
+2. Observa el comportamiento.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clickear el boton de atras solo una vez. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">La pagina regresa correctamente a donde se selecciono el pin. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">La pagina regresa al feed principal mostrando las mismas imagenes y teniendo mismo limite. </t>
+  </si>
+  <si>
+    <t>CP07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.En el feed, hacer clic derecho sobre un pin.
+2. Seleccionar “Abrir enlace en una nueva pestaña”.
+3. Cambiar a esa pestaña.
+4. Observar el comportamiento de la pestana independiente. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validar la respuesta desde otra pestaña. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abrir el pin para otra pestaña. </t>
+  </si>
+  <si>
+    <t>El pin se abre sin ningún error.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El pin se abre correctamente en la pestaña exterior y a la vez muestra sugerencias del mismo. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baja </t>
+  </si>
+  <si>
+    <t>CP08</t>
+  </si>
+  <si>
+    <t>1. En el feed (no dentro de un pin), reducir manualmente el tamaño de la ventana arrastrando desde una esquina.
+2. Hacerla más angosta.
+3. Luego volver a ampliarla.
+4. Observar durante el proceso.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verificar la adaptabilidad de la feed. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reducir el tamaño de la pestaña. </t>
+  </si>
+  <si>
+    <t>El layout se adapta correctamente al redimensionar la ventana. Se observa breve pantalla en blanco (2–3 segundos) mientras se reorganizan las imágenes, sin afectar funcionalidad.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acomodación automatica de las imágenes mientras se minimiza. </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="14"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -95,8 +293,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -431,41 +638,545 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA54B7BA-EFE9-4C27-A1EF-EDC1F716815F}">
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:O21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="2" max="2" width="17.85546875" customWidth="1"/>
     <col min="3" max="3" width="18.7109375" customWidth="1"/>
-    <col min="5" max="5" width="20.42578125" customWidth="1"/>
-    <col min="6" max="6" width="18.85546875" customWidth="1"/>
+    <col min="4" max="4" width="21.42578125" customWidth="1"/>
+    <col min="5" max="5" width="31.5703125" customWidth="1"/>
+    <col min="6" max="6" width="27.7109375" customWidth="1"/>
+    <col min="7" max="7" width="28.28515625" customWidth="1"/>
+    <col min="8" max="8" width="13.7109375" customWidth="1"/>
+    <col min="9" max="9" width="16.7109375" customWidth="1"/>
+    <col min="11" max="11" width="20.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:15" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" s="2" t="s">
         <v>7</v>
       </c>
+      <c r="J1" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" ht="90" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
+      <c r="N2" s="1"/>
+      <c r="O2" s="1"/>
+    </row>
+    <row r="3" spans="1:15" ht="120" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="K3" s="1"/>
+      <c r="L3" s="1"/>
+      <c r="M3" s="1"/>
+      <c r="N3" s="1"/>
+      <c r="O3" s="1"/>
+    </row>
+    <row r="4" spans="1:15" ht="90" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="L4" s="1"/>
+      <c r="M4" s="1"/>
+      <c r="N4" s="1"/>
+      <c r="O4" s="1"/>
+    </row>
+    <row r="5" spans="1:15" ht="105" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="K5" s="1"/>
+      <c r="L5" s="1"/>
+      <c r="M5" s="1"/>
+      <c r="N5" s="1"/>
+      <c r="O5" s="1"/>
+    </row>
+    <row r="6" spans="1:15" ht="75" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
+      <c r="N6" s="1"/>
+      <c r="O6" s="1"/>
+    </row>
+    <row r="7" spans="1:15" ht="75" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B7" s="1"/>
+      <c r="C7" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="K7" s="1"/>
+      <c r="L7" s="1"/>
+      <c r="M7" s="1"/>
+      <c r="N7" s="1"/>
+      <c r="O7" s="1"/>
+    </row>
+    <row r="8" spans="1:15" ht="105" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B8" s="1"/>
+      <c r="C8" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="K8" s="1"/>
+      <c r="L8" s="1"/>
+      <c r="M8" s="1"/>
+      <c r="N8" s="1"/>
+      <c r="O8" s="1"/>
+    </row>
+    <row r="9" spans="1:15" ht="120" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B9" s="1"/>
+      <c r="C9" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="K9" s="1"/>
+      <c r="L9" s="1"/>
+      <c r="M9" s="1"/>
+      <c r="N9" s="1"/>
+      <c r="O9" s="1"/>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A10" s="1"/>
+      <c r="B10" s="1"/>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
+      <c r="G10" s="1"/>
+      <c r="H10" s="1"/>
+      <c r="I10" s="1"/>
+      <c r="J10" s="1"/>
+      <c r="K10" s="1"/>
+      <c r="L10" s="1"/>
+      <c r="M10" s="1"/>
+      <c r="N10" s="1"/>
+      <c r="O10" s="1"/>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A11" s="1"/>
+      <c r="B11" s="1"/>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
+      <c r="G11" s="1"/>
+      <c r="H11" s="1"/>
+      <c r="I11" s="1"/>
+      <c r="J11" s="1"/>
+      <c r="K11" s="1"/>
+      <c r="L11" s="1"/>
+      <c r="M11" s="1"/>
+      <c r="N11" s="1"/>
+      <c r="O11" s="1"/>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A12" s="1"/>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
+      <c r="G12" s="1"/>
+      <c r="H12" s="1"/>
+      <c r="I12" s="1"/>
+      <c r="J12" s="1"/>
+      <c r="K12" s="1"/>
+      <c r="L12" s="1"/>
+      <c r="M12" s="1"/>
+      <c r="N12" s="1"/>
+      <c r="O12" s="1"/>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A13" s="1"/>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
+      <c r="G13" s="1"/>
+      <c r="H13" s="1"/>
+      <c r="I13" s="1"/>
+      <c r="J13" s="1"/>
+      <c r="K13" s="1"/>
+      <c r="L13" s="1"/>
+      <c r="M13" s="1"/>
+      <c r="N13" s="1"/>
+      <c r="O13" s="1"/>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A14" s="1"/>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
+      <c r="G14" s="1"/>
+      <c r="H14" s="1"/>
+      <c r="I14" s="1"/>
+      <c r="J14" s="1"/>
+      <c r="K14" s="1"/>
+      <c r="L14" s="1"/>
+      <c r="M14" s="1"/>
+      <c r="N14" s="1"/>
+      <c r="O14" s="1"/>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A15" s="1"/>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
+      <c r="G15" s="1"/>
+      <c r="H15" s="1"/>
+      <c r="I15" s="1"/>
+      <c r="J15" s="1"/>
+      <c r="K15" s="1"/>
+      <c r="L15" s="1"/>
+      <c r="M15" s="1"/>
+      <c r="N15" s="1"/>
+      <c r="O15" s="1"/>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A16" s="1"/>
+      <c r="B16" s="1"/>
+      <c r="C16" s="1"/>
+      <c r="D16" s="1"/>
+      <c r="E16" s="1"/>
+      <c r="F16" s="1"/>
+      <c r="G16" s="1"/>
+      <c r="H16" s="1"/>
+      <c r="I16" s="1"/>
+      <c r="J16" s="1"/>
+      <c r="K16" s="1"/>
+      <c r="L16" s="1"/>
+      <c r="M16" s="1"/>
+      <c r="N16" s="1"/>
+      <c r="O16" s="1"/>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A17" s="1"/>
+      <c r="B17" s="1"/>
+      <c r="C17" s="1"/>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+      <c r="F17" s="1"/>
+      <c r="G17" s="1"/>
+      <c r="H17" s="1"/>
+      <c r="I17" s="1"/>
+      <c r="J17" s="1"/>
+      <c r="K17" s="1"/>
+      <c r="L17" s="1"/>
+      <c r="M17" s="1"/>
+      <c r="N17" s="1"/>
+      <c r="O17" s="1"/>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A18" s="1"/>
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+      <c r="F18" s="1"/>
+      <c r="G18" s="1"/>
+      <c r="H18" s="1"/>
+      <c r="I18" s="1"/>
+      <c r="J18" s="1"/>
+      <c r="K18" s="1"/>
+      <c r="L18" s="1"/>
+      <c r="M18" s="1"/>
+      <c r="N18" s="1"/>
+      <c r="O18" s="1"/>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A19" s="1"/>
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+      <c r="F19" s="1"/>
+      <c r="G19" s="1"/>
+      <c r="H19" s="1"/>
+      <c r="I19" s="1"/>
+      <c r="J19" s="1"/>
+      <c r="K19" s="1"/>
+      <c r="L19" s="1"/>
+      <c r="M19" s="1"/>
+      <c r="N19" s="1"/>
+      <c r="O19" s="1"/>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A20" s="1"/>
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+      <c r="F20" s="1"/>
+      <c r="G20" s="1"/>
+      <c r="H20" s="1"/>
+      <c r="I20" s="1"/>
+      <c r="J20" s="1"/>
+      <c r="K20" s="1"/>
+      <c r="L20" s="1"/>
+      <c r="M20" s="1"/>
+      <c r="N20" s="1"/>
+      <c r="O20" s="1"/>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A21" s="1"/>
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+      <c r="F21" s="1"/>
+      <c r="G21" s="1"/>
+      <c r="H21" s="1"/>
+      <c r="I21" s="1"/>
+      <c r="J21" s="1"/>
+      <c r="K21" s="1"/>
+      <c r="L21" s="1"/>
+      <c r="M21" s="1"/>
+      <c r="N21" s="1"/>
+      <c r="O21" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Ejecuto bloque Busqueda y registro resultados con 2 bugs detectados
</commit_message>
<xml_diff>
--- a/casos_de_prueba/matriz_pruebas.xlsx
+++ b/casos_de_prueba/matriz_pruebas.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USUARIO\Desktop\ProyectoFinal-QA-Scarleth\casos_de_prueba\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73F084C9-E377-426F-8528-781A64ABABC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35223DCA-8A55-406C-89C9-7F3D06ECC9CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{5FF4DDCA-2057-4105-B76A-F7B3AA90F74B}"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="Casos-de-prueba" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="112">
   <si>
     <t>ID</t>
   </si>
@@ -241,13 +241,189 @@
   </si>
   <si>
     <t xml:space="preserve">Acomodación automatica de las imágenes mientras se minimiza. </t>
+  </si>
+  <si>
+    <t>CP09</t>
+  </si>
+  <si>
+    <t>Búsqueda</t>
+  </si>
+  <si>
+    <t>Confirmar que la búsqueda devuelve resultados relevantes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filtrar busqueda con palabra "decoración". </t>
+  </si>
+  <si>
+    <t>1. En Pinterest, ubicar la barra de búsqueda.
+2. Escribir: decoración (sin comillas).
+3. Presionar Enter.</t>
+  </si>
+  <si>
+    <t>La página muestra resultados según la palabra.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mostró resultado según filtro y sugirió según temática. </t>
+  </si>
+  <si>
+    <t>CP10</t>
+  </si>
+  <si>
+    <t>Validar qué ocurre cuando el usuario intenta buscar sin escribir nada.</t>
+  </si>
+  <si>
+    <t>El campo de busqueda debe estar vacío.</t>
+  </si>
+  <si>
+    <t>1. Hacer clic en la barra de búsqueda.
+2. Borrar cualquier texto si lo hay.
+3. Dejar el campo vacío.
+4. Presionar Enter.</t>
+  </si>
+  <si>
+    <t>La página da mensaje de feedback para escribir algo en la búsqueda.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La página no reacciona, no lanza mensaje de colocar algo en la busqueda. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fail </t>
+  </si>
+  <si>
+    <t>CP11</t>
+  </si>
+  <si>
+    <t>Validar el sistema caracteres no alfabéticos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Utilizar los caracteres no alfabéticos. </t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. Ir a la barra de buesqueda.                2. Escribir solo </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">@#$%   </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">                         3. Presionar enter</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Mensaje de no lectura de la búsqueda. </t>
+  </si>
+  <si>
+    <t>La página lanza una serie de imágenes.</t>
+  </si>
+  <si>
+    <t>CP12</t>
+  </si>
+  <si>
+    <t>Validar la respuesta del sistema cuando no hay resultados.</t>
+  </si>
+  <si>
+    <t>1. Ir a la barra de búsqueda.
+2. Escribir un término “imposible”, por ejemplo:
+qwertyuiopasdfghjklzxcvbnm123
+3. Presionar Enter.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ejecutar con el término dado. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mensaje de error o de sugerencias para utilizar otro término. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lanza una diversidad de imágenes y esta vez, tiro el mensaje de Longin como respuesta. </t>
+  </si>
+  <si>
+    <t>CP13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validar la similitud de los resultados con la misma palabra en mayúsculas y miniculas. </t>
+  </si>
+  <si>
+    <t>Utilizar la palabra (decoración / DECORACIÓN / DeCoRaCiÓn).</t>
+  </si>
+  <si>
+    <t>En cada paso se deben observar los resultados obtenidos.                            1. Buscar con decoración.                      2. Buscar DESCORACIÓN                      3. Buscar con DeCoRaCiÓn.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Similutd en las sugerencias con las tres búsquedas. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Las imágenes de los resultados fueron similares / coherentes con el filtro. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Una de las imágenes mostrada en el filtro se repitió las tres busquedas. </t>
+  </si>
+  <si>
+    <t>CP14</t>
+  </si>
+  <si>
+    <t>Ver si el sistema maneja correctamente cambios rápidos de término sin dañar los resultados.</t>
+  </si>
+  <si>
+    <t>Hacerlo con intervalos cortos (1–2 segundos entre cada búsqueda).</t>
+  </si>
+  <si>
+    <t>1. Escribir: decoración - Enter.
+2. Inmediatamente cambiar a: cocina - Enter.
+3. Luego cambiar rápido a: viajes - Enter.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carga correctamente cada término, mostrando las imágenes correspondientes a los mismos. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Muestra completamente y correctamente los resultados. </t>
+  </si>
+  <si>
+    <t>CP15</t>
+  </si>
+  <si>
+    <t>Validar qué ocurre cuando se borra el término después de haber buscado algo.</t>
+  </si>
+  <si>
+    <t>1. Buscar: decoración
+2. Cuando carguen resultados, hacer clic en la barra de búsqueda
+3. Borrar el texto completamente
+4. No presionar Enter aún
+5. Observar qué ocurre
+6. Luego presionar Enter</t>
+  </si>
+  <si>
+    <t>Al borrar el término de búsqueda, el sistema mantiene los resultados anteriores. Al presionar Enter con campo vacío no se ejecuta nueva acción ni se muestra mensaje de validación.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mensaje de colocar al menos 1 término para hacer búsqueda. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mantiene el resultado aún si un termino. </t>
+  </si>
+  <si>
+    <t>Borrar y clickear enter sin termino en la busqueda.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -267,6 +443,14 @@
       <b/>
       <i/>
       <sz val="14"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -293,7 +477,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -303,6 +487,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -638,7 +825,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA54B7BA-EFE9-4C27-A1EF-EDC1F716815F}">
-  <dimension ref="A1:O21"/>
+  <dimension ref="A1:O34"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="17.85546875" customWidth="1"/>
@@ -724,7 +911,7 @@
       <c r="N2" s="1"/>
       <c r="O2" s="1"/>
     </row>
-    <row r="3" spans="1:15" ht="120" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" ht="75" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>18</v>
       </c>
@@ -759,7 +946,7 @@
       <c r="N3" s="1"/>
       <c r="O3" s="1"/>
     </row>
-    <row r="4" spans="1:15" ht="90" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>26</v>
       </c>
@@ -796,7 +983,7 @@
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
     </row>
-    <row r="5" spans="1:15" ht="105" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" ht="75" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>34</v>
       </c>
@@ -866,7 +1053,7 @@
       <c r="N6" s="1"/>
       <c r="O6" s="1"/>
     </row>
-    <row r="7" spans="1:15" ht="75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>47</v>
       </c>
@@ -971,209 +1158,523 @@
       <c r="N9" s="1"/>
       <c r="O9" s="1"/>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A10" s="1"/>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
-      <c r="F10" s="1"/>
-      <c r="G10" s="1"/>
-      <c r="H10" s="1"/>
-      <c r="I10" s="1"/>
-      <c r="J10" s="1"/>
+    <row r="10" spans="1:15" ht="75" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>17</v>
+      </c>
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
       <c r="M10" s="1"/>
       <c r="N10" s="1"/>
       <c r="O10" s="1"/>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A11" s="1"/>
+    <row r="11" spans="1:15" ht="75" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>73</v>
+      </c>
       <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
-      <c r="F11" s="1"/>
-      <c r="G11" s="1"/>
-      <c r="H11" s="1"/>
-      <c r="I11" s="1"/>
-      <c r="J11" s="1"/>
+      <c r="C11" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>79</v>
+      </c>
       <c r="K11" s="1"/>
       <c r="L11" s="1"/>
       <c r="M11" s="1"/>
       <c r="N11" s="1"/>
       <c r="O11" s="1"/>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A12" s="1"/>
+    <row r="12" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>80</v>
+      </c>
       <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
-      <c r="F12" s="1"/>
-      <c r="G12" s="1"/>
-      <c r="H12" s="1"/>
-      <c r="I12" s="1"/>
-      <c r="J12" s="1"/>
+      <c r="C12" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J12" s="1" t="s">
+        <v>79</v>
+      </c>
       <c r="K12" s="1"/>
       <c r="L12" s="1"/>
       <c r="M12" s="1"/>
       <c r="N12" s="1"/>
       <c r="O12" s="1"/>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A13" s="1"/>
+    <row r="13" spans="1:15" ht="75" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>86</v>
+      </c>
       <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
-      <c r="F13" s="1"/>
-      <c r="G13" s="1"/>
-      <c r="H13" s="1"/>
-      <c r="I13" s="1"/>
-      <c r="J13" s="1"/>
+      <c r="C13" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I13" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="J13" s="1" t="s">
+        <v>17</v>
+      </c>
       <c r="K13" s="1"/>
       <c r="L13" s="1"/>
       <c r="M13" s="1"/>
       <c r="N13" s="1"/>
       <c r="O13" s="1"/>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" s="1"/>
+    <row r="14" spans="1:15" ht="90" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>92</v>
+      </c>
       <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
-      <c r="F14" s="1"/>
-      <c r="G14" s="1"/>
-      <c r="H14" s="1"/>
-      <c r="I14" s="1"/>
-      <c r="J14" s="1"/>
-      <c r="K14" s="1"/>
+      <c r="C14" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J14" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="K14" s="1" t="s">
+        <v>98</v>
+      </c>
       <c r="L14" s="1"/>
       <c r="M14" s="1"/>
       <c r="N14" s="1"/>
       <c r="O14" s="1"/>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" s="1"/>
+    <row r="15" spans="1:15" ht="90" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>99</v>
+      </c>
       <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
-      <c r="F15" s="1"/>
-      <c r="G15" s="1"/>
-      <c r="H15" s="1"/>
-      <c r="I15" s="1"/>
-      <c r="J15" s="1"/>
+      <c r="C15" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I15" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J15" s="1" t="s">
+        <v>17</v>
+      </c>
       <c r="K15" s="1"/>
       <c r="L15" s="1"/>
       <c r="M15" s="1"/>
       <c r="N15" s="1"/>
       <c r="O15" s="1"/>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" s="1"/>
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
-      <c r="D16" s="1"/>
-      <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
-      <c r="G16" s="1"/>
-      <c r="H16" s="1"/>
-      <c r="I16" s="1"/>
-      <c r="J16" s="1"/>
-      <c r="K16" s="1"/>
-      <c r="L16" s="1"/>
+    <row r="16" spans="1:15" ht="150" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="B16" s="4"/>
+      <c r="C16" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="H16" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="I16" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="J16" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="K16" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="L16" s="4"/>
       <c r="M16" s="1"/>
       <c r="N16" s="1"/>
       <c r="O16" s="1"/>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A17" s="1"/>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1"/>
-      <c r="E17" s="1"/>
-      <c r="F17" s="1"/>
-      <c r="G17" s="1"/>
-      <c r="H17" s="1"/>
-      <c r="I17" s="1"/>
-      <c r="J17" s="1"/>
-      <c r="K17" s="1"/>
-      <c r="L17" s="1"/>
+      <c r="A17" s="4"/>
+      <c r="B17" s="4"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4"/>
+      <c r="F17" s="4"/>
+      <c r="G17" s="4"/>
+      <c r="H17" s="4"/>
+      <c r="I17" s="4"/>
+      <c r="J17" s="4"/>
+      <c r="K17" s="4"/>
+      <c r="L17" s="4"/>
       <c r="M17" s="1"/>
       <c r="N17" s="1"/>
       <c r="O17" s="1"/>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A18" s="1"/>
-      <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
-      <c r="D18" s="1"/>
-      <c r="E18" s="1"/>
-      <c r="F18" s="1"/>
-      <c r="G18" s="1"/>
-      <c r="H18" s="1"/>
-      <c r="I18" s="1"/>
-      <c r="J18" s="1"/>
-      <c r="K18" s="1"/>
-      <c r="L18" s="1"/>
+      <c r="A18" s="4"/>
+      <c r="B18" s="4"/>
+      <c r="C18" s="4"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4"/>
+      <c r="F18" s="4"/>
+      <c r="G18" s="4"/>
+      <c r="H18" s="4"/>
+      <c r="I18" s="4"/>
+      <c r="J18" s="4"/>
+      <c r="K18" s="4"/>
+      <c r="L18" s="4"/>
       <c r="M18" s="1"/>
       <c r="N18" s="1"/>
       <c r="O18" s="1"/>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A19" s="1"/>
-      <c r="B19" s="1"/>
-      <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
-      <c r="E19" s="1"/>
-      <c r="F19" s="1"/>
-      <c r="G19" s="1"/>
-      <c r="H19" s="1"/>
-      <c r="I19" s="1"/>
-      <c r="J19" s="1"/>
-      <c r="K19" s="1"/>
-      <c r="L19" s="1"/>
+      <c r="A19" s="4"/>
+      <c r="B19" s="4"/>
+      <c r="C19" s="4"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4"/>
+      <c r="F19" s="4"/>
+      <c r="G19" s="4"/>
+      <c r="H19" s="4"/>
+      <c r="I19" s="4"/>
+      <c r="J19" s="4"/>
+      <c r="K19" s="4"/>
+      <c r="L19" s="4"/>
       <c r="M19" s="1"/>
       <c r="N19" s="1"/>
       <c r="O19" s="1"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A20" s="1"/>
-      <c r="B20" s="1"/>
-      <c r="C20" s="1"/>
-      <c r="D20" s="1"/>
-      <c r="E20" s="1"/>
-      <c r="F20" s="1"/>
-      <c r="G20" s="1"/>
-      <c r="H20" s="1"/>
-      <c r="I20" s="1"/>
-      <c r="J20" s="1"/>
-      <c r="K20" s="1"/>
-      <c r="L20" s="1"/>
+      <c r="A20" s="4"/>
+      <c r="B20" s="4"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="4"/>
+      <c r="F20" s="4"/>
+      <c r="G20" s="4"/>
+      <c r="H20" s="4"/>
+      <c r="I20" s="4"/>
+      <c r="J20" s="4"/>
+      <c r="K20" s="4"/>
+      <c r="L20" s="4"/>
       <c r="M20" s="1"/>
       <c r="N20" s="1"/>
       <c r="O20" s="1"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21" s="1"/>
-      <c r="B21" s="1"/>
-      <c r="C21" s="1"/>
-      <c r="D21" s="1"/>
-      <c r="E21" s="1"/>
-      <c r="F21" s="1"/>
-      <c r="G21" s="1"/>
-      <c r="H21" s="1"/>
-      <c r="I21" s="1"/>
-      <c r="J21" s="1"/>
-      <c r="K21" s="1"/>
-      <c r="L21" s="1"/>
+      <c r="A21" s="4"/>
+      <c r="B21" s="4"/>
+      <c r="C21" s="4"/>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4"/>
+      <c r="F21" s="4"/>
+      <c r="G21" s="4"/>
+      <c r="H21" s="4"/>
+      <c r="I21" s="4"/>
+      <c r="J21" s="4"/>
+      <c r="K21" s="4"/>
+      <c r="L21" s="4"/>
       <c r="M21" s="1"/>
       <c r="N21" s="1"/>
       <c r="O21" s="1"/>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A22" s="4"/>
+      <c r="B22" s="4"/>
+      <c r="C22" s="4"/>
+      <c r="D22" s="4"/>
+      <c r="E22" s="4"/>
+      <c r="F22" s="4"/>
+      <c r="G22" s="4"/>
+      <c r="H22" s="4"/>
+      <c r="I22" s="4"/>
+      <c r="J22" s="4"/>
+      <c r="K22" s="4"/>
+      <c r="L22" s="4"/>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A23" s="4"/>
+      <c r="B23" s="4"/>
+      <c r="C23" s="4"/>
+      <c r="D23" s="4"/>
+      <c r="E23" s="4"/>
+      <c r="F23" s="4"/>
+      <c r="G23" s="4"/>
+      <c r="H23" s="4"/>
+      <c r="I23" s="4"/>
+      <c r="J23" s="4"/>
+      <c r="K23" s="4"/>
+      <c r="L23" s="4"/>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A24" s="4"/>
+      <c r="B24" s="4"/>
+      <c r="C24" s="4"/>
+      <c r="D24" s="4"/>
+      <c r="E24" s="4"/>
+      <c r="F24" s="4"/>
+      <c r="G24" s="4"/>
+      <c r="H24" s="4"/>
+      <c r="I24" s="4"/>
+      <c r="J24" s="4"/>
+      <c r="K24" s="4"/>
+      <c r="L24" s="4"/>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A25" s="4"/>
+      <c r="B25" s="4"/>
+      <c r="C25" s="4"/>
+      <c r="D25" s="4"/>
+      <c r="E25" s="4"/>
+      <c r="F25" s="4"/>
+      <c r="G25" s="4"/>
+      <c r="H25" s="4"/>
+      <c r="I25" s="4"/>
+      <c r="J25" s="4"/>
+      <c r="K25" s="4"/>
+      <c r="L25" s="4"/>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A26" s="4"/>
+      <c r="B26" s="4"/>
+      <c r="C26" s="4"/>
+      <c r="D26" s="4"/>
+      <c r="E26" s="4"/>
+      <c r="F26" s="4"/>
+      <c r="G26" s="4"/>
+      <c r="H26" s="4"/>
+      <c r="I26" s="4"/>
+      <c r="J26" s="4"/>
+      <c r="K26" s="4"/>
+      <c r="L26" s="4"/>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A27" s="4"/>
+      <c r="B27" s="4"/>
+      <c r="C27" s="4"/>
+      <c r="D27" s="4"/>
+      <c r="E27" s="4"/>
+      <c r="F27" s="4"/>
+      <c r="G27" s="4"/>
+      <c r="H27" s="4"/>
+      <c r="I27" s="4"/>
+      <c r="J27" s="4"/>
+      <c r="K27" s="4"/>
+      <c r="L27" s="4"/>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A28" s="4"/>
+      <c r="B28" s="4"/>
+      <c r="C28" s="4"/>
+      <c r="D28" s="4"/>
+      <c r="E28" s="4"/>
+      <c r="F28" s="4"/>
+      <c r="G28" s="4"/>
+      <c r="H28" s="4"/>
+      <c r="I28" s="4"/>
+      <c r="J28" s="4"/>
+      <c r="K28" s="4"/>
+      <c r="L28" s="4"/>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A29" s="4"/>
+      <c r="B29" s="4"/>
+      <c r="C29" s="4"/>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4"/>
+      <c r="F29" s="4"/>
+      <c r="G29" s="4"/>
+      <c r="H29" s="4"/>
+      <c r="I29" s="4"/>
+      <c r="J29" s="4"/>
+      <c r="K29" s="4"/>
+      <c r="L29" s="4"/>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A30" s="4"/>
+      <c r="B30" s="4"/>
+      <c r="C30" s="4"/>
+      <c r="D30" s="4"/>
+      <c r="E30" s="4"/>
+      <c r="F30" s="4"/>
+      <c r="G30" s="4"/>
+      <c r="H30" s="4"/>
+      <c r="I30" s="4"/>
+      <c r="J30" s="4"/>
+      <c r="K30" s="4"/>
+      <c r="L30" s="4"/>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A31" s="4"/>
+      <c r="B31" s="4"/>
+      <c r="C31" s="4"/>
+      <c r="D31" s="4"/>
+      <c r="E31" s="4"/>
+      <c r="F31" s="4"/>
+      <c r="G31" s="4"/>
+      <c r="H31" s="4"/>
+      <c r="I31" s="4"/>
+      <c r="J31" s="4"/>
+      <c r="K31" s="4"/>
+      <c r="L31" s="4"/>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A32" s="4"/>
+      <c r="B32" s="4"/>
+      <c r="C32" s="4"/>
+      <c r="D32" s="4"/>
+      <c r="E32" s="4"/>
+      <c r="F32" s="4"/>
+      <c r="G32" s="4"/>
+      <c r="H32" s="4"/>
+      <c r="I32" s="4"/>
+      <c r="J32" s="4"/>
+      <c r="K32" s="4"/>
+      <c r="L32" s="4"/>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A33" s="4"/>
+      <c r="B33" s="4"/>
+      <c r="C33" s="4"/>
+      <c r="D33" s="4"/>
+      <c r="E33" s="4"/>
+      <c r="F33" s="4"/>
+      <c r="G33" s="4"/>
+      <c r="H33" s="4"/>
+      <c r="I33" s="4"/>
+      <c r="J33" s="4"/>
+      <c r="K33" s="4"/>
+      <c r="L33" s="4"/>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A34" s="4"/>
+      <c r="B34" s="4"/>
+      <c r="C34" s="4"/>
+      <c r="D34" s="4"/>
+      <c r="E34" s="4"/>
+      <c r="F34" s="4"/>
+      <c r="G34" s="4"/>
+      <c r="H34" s="4"/>
+      <c r="I34" s="4"/>
+      <c r="J34" s="4"/>
+      <c r="K34" s="4"/>
+      <c r="L34" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
agrego evidencia en video prueba responsive rotacion movil
</commit_message>
<xml_diff>
--- a/casos_de_prueba/matriz_pruebas.xlsx
+++ b/casos_de_prueba/matriz_pruebas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USUARIO\Desktop\ProyectoFinal-QA-Scarleth\casos_de_prueba\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D5A1A26-F28C-48EE-AEDB-85C2A8DA1D76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E393E5C5-F6EB-4B53-89B5-37F70A625F33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{5FF4DDCA-2057-4105-B76A-F7B3AA90F74B}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="152">
   <si>
     <t>ID</t>
   </si>
@@ -459,6 +459,96 @@
   </si>
   <si>
     <t>Error tipo XML</t>
+  </si>
+  <si>
+    <t>CP18</t>
+  </si>
+  <si>
+    <t>Validar que la URL del pin pueda copiarse correctamente y funcione al abrirla.</t>
+  </si>
+  <si>
+    <t>1. Abrir un pin cualquiera.
+2. Copiar la URL directamente desde la barra del navegador.
+3. Abre una nueva pestaña.
+4. Pegar la URL copiada.
+5. Presionar Enter.</t>
+  </si>
+  <si>
+    <t>El pin debe abrir correctamente mostrando el mismo contenido.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Muestra el mismo contenido que el pin fuente. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seleccionar el enlace que tiene el pin. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abrir una nueva ventana para ver resultados del pin. </t>
+  </si>
+  <si>
+    <t>CP19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validar los detalles de un pin sugerido. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Navegar con un pin sugerido (no principal). </t>
+  </si>
+  <si>
+    <t>1. Abrir un pin cualquiera.
+2. En la sección de pines sugeridos (lado derecho o debajo), hacer clic en uno diferente.
+3.Observar el cambio.</t>
+  </si>
+  <si>
+    <t>Al abrir un pin sugerido y Hacer scroll, se muestra un tablero de destacados, modificando ligeramente la disposición visual sin afectar funcionalidad.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La información e imagen cambia. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fluye correctamente la información del otro pin. </t>
+  </si>
+  <si>
+    <t>CP20</t>
+  </si>
+  <si>
+    <t>Validar estabilidad al hacer scroll dentro del detalle.</t>
+  </si>
+  <si>
+    <t>1. Abrir un pin.
+2. Hacer scroll hacia abajo hasta donde cargue contenido adicional.
+3. Observar durante la carga.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hacer scroll continuo. </t>
+  </si>
+  <si>
+    <t>Durante el scroll se cargan pines relacionados. Se observa ampliación de temática dentro de la categoría belleza. Algunos pines se repiten, sin afectar funcionalidad.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El contenido adicional fluye correctamente sin repetir contenido, dando sugerencias y sin quedar en blanco o bloquear el scroll. </t>
+  </si>
+  <si>
+    <t>Al ingresar con un pin, los demas que aparecen van tomando concordancia en cuanto a la tematica del pin principal.</t>
+  </si>
+  <si>
+    <t>CP21</t>
+  </si>
+  <si>
+    <t>Validar estabilidad cuando el usuario navega rápidamente entre pines sugeridos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Repetir la navegación entre 3-4 veces. </t>
+  </si>
+  <si>
+    <t>1. Abrir un pin.                                                2. Hacer clic en un pin sugerido.
+3. Inmediatamente hacer clic en otro sugerido.                                                           4. Repetir 3–4 veces rápido.</t>
+  </si>
+  <si>
+    <t>La página tiene estabilidad en cargar información de cada pin seleccionado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No hubo pantalla en blanco por lo que página cargó correctamente cada pin nuevo. </t>
   </si>
 </sst>
 </file>
@@ -499,12 +589,30 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.89999084444715716"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -519,7 +627,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -532,6 +640,19 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -917,107 +1038,107 @@
       </c>
     </row>
     <row r="2" spans="1:15" ht="90" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="F2" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="G2" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="H2" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="I2" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="J2" s="1" t="s">
+      <c r="I2" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="J2" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="K2" s="1"/>
+      <c r="K2" s="9"/>
       <c r="L2" s="1"/>
       <c r="M2" s="1"/>
       <c r="N2" s="1"/>
       <c r="O2" s="1"/>
     </row>
     <row r="3" spans="1:15" ht="75" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1" t="s">
+      <c r="B3" s="9"/>
+      <c r="C3" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E3" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="F3" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="G3" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="H3" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="I3" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="J3" s="1" t="s">
+      <c r="J3" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="K3" s="1"/>
+      <c r="K3" s="9"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
       <c r="N3" s="1"/>
       <c r="O3" s="1"/>
     </row>
     <row r="4" spans="1:15" ht="60" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1" t="s">
+      <c r="B4" s="9"/>
+      <c r="C4" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D4" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="E4" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="F4" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="G4" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="H4" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="I4" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="J4" s="1" t="s">
+      <c r="I4" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="J4" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="K4" s="1" t="s">
+      <c r="K4" s="9" t="s">
         <v>33</v>
       </c>
       <c r="L4" s="1"/>
@@ -1026,352 +1147,352 @@
       <c r="O4" s="1"/>
     </row>
     <row r="5" spans="1:15" ht="75" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1" t="s">
+      <c r="B5" s="9"/>
+      <c r="C5" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D5" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="E5" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="F5" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="G5" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="H5" s="1" t="s">
+      <c r="H5" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="I5" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="J5" s="1" t="s">
+      <c r="I5" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="J5" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="K5" s="1"/>
+      <c r="K5" s="9"/>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
       <c r="N5" s="1"/>
       <c r="O5" s="1"/>
     </row>
     <row r="6" spans="1:15" ht="75" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1" t="s">
+      <c r="B6" s="9"/>
+      <c r="C6" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F6" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="G6" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="H6" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="I6" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="J6" s="1" t="s">
+      <c r="I6" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="J6" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="K6" s="1"/>
+      <c r="K6" s="9"/>
       <c r="L6" s="1"/>
       <c r="M6" s="1"/>
       <c r="N6" s="1"/>
       <c r="O6" s="1"/>
     </row>
     <row r="7" spans="1:15" ht="60" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1" t="s">
+      <c r="B7" s="9"/>
+      <c r="C7" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="D7" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="E7" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="F7" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="G7" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="H7" s="1" t="s">
+      <c r="H7" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="I7" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="J7" s="1" t="s">
+      <c r="I7" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="J7" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="K7" s="1"/>
+      <c r="K7" s="9"/>
       <c r="L7" s="1"/>
       <c r="M7" s="1"/>
       <c r="N7" s="1"/>
       <c r="O7" s="1"/>
     </row>
     <row r="8" spans="1:15" ht="105" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1" t="s">
+      <c r="B8" s="9"/>
+      <c r="C8" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="D8" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="E8" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="F8" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="G8" s="1" t="s">
+      <c r="G8" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="H8" s="1" t="s">
+      <c r="H8" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="I8" s="1" t="s">
+      <c r="I8" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="J8" s="1" t="s">
+      <c r="J8" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="K8" s="1"/>
+      <c r="K8" s="9"/>
       <c r="L8" s="1"/>
       <c r="M8" s="1"/>
       <c r="N8" s="1"/>
       <c r="O8" s="1"/>
     </row>
     <row r="9" spans="1:15" ht="120" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1" t="s">
+      <c r="B9" s="9"/>
+      <c r="C9" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="D9" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="E9" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="F9" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="G9" s="1" t="s">
+      <c r="G9" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="H9" s="1" t="s">
+      <c r="H9" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="I9" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="J9" s="1" t="s">
+      <c r="I9" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="J9" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="K9" s="1"/>
+      <c r="K9" s="9"/>
       <c r="L9" s="1"/>
       <c r="M9" s="1"/>
       <c r="N9" s="1"/>
       <c r="O9" s="1"/>
     </row>
     <row r="10" spans="1:15" ht="75" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
+      <c r="A10" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="D10" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="E10" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="F10" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="G10" s="1" t="s">
+      <c r="G10" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="H10" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="I10" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="J10" s="1" t="s">
+      <c r="H10" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="I10" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="J10" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="K10" s="1"/>
+      <c r="K10" s="7"/>
       <c r="L10" s="1"/>
       <c r="M10" s="1"/>
       <c r="N10" s="1"/>
       <c r="O10" s="1"/>
     </row>
     <row r="11" spans="1:15" ht="75" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
+      <c r="A11" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1" t="s">
+      <c r="B11" s="7"/>
+      <c r="C11" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="D11" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="E11" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="F11" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="G11" s="1" t="s">
+      <c r="G11" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="H11" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="I11" s="1" t="s">
+      <c r="H11" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="I11" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="J11" s="1" t="s">
+      <c r="J11" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="K11" s="1"/>
+      <c r="K11" s="7"/>
       <c r="L11" s="1"/>
       <c r="M11" s="1"/>
       <c r="N11" s="1"/>
       <c r="O11" s="1"/>
     </row>
     <row r="12" spans="1:15" ht="45" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
+      <c r="A12" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1" t="s">
+      <c r="B12" s="7"/>
+      <c r="C12" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="D12" s="1" t="s">
+      <c r="D12" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="E12" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="F12" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="G12" s="1" t="s">
+      <c r="G12" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="H12" s="1" t="s">
+      <c r="H12" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="I12" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="J12" s="1" t="s">
+      <c r="I12" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="J12" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="K12" s="1"/>
+      <c r="K12" s="7"/>
       <c r="L12" s="1"/>
       <c r="M12" s="1"/>
       <c r="N12" s="1"/>
       <c r="O12" s="1"/>
     </row>
     <row r="13" spans="1:15" ht="75" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
+      <c r="A13" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1" t="s">
+      <c r="B13" s="7"/>
+      <c r="C13" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="D13" s="1" t="s">
+      <c r="D13" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="E13" s="1" t="s">
+      <c r="E13" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="F13" s="1" t="s">
+      <c r="F13" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="G13" s="1" t="s">
+      <c r="G13" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="H13" s="1" t="s">
+      <c r="H13" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="I13" s="1" t="s">
+      <c r="I13" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="J13" s="1" t="s">
+      <c r="J13" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="K13" s="1"/>
+      <c r="K13" s="7"/>
       <c r="L13" s="1"/>
       <c r="M13" s="1"/>
       <c r="N13" s="1"/>
       <c r="O13" s="1"/>
     </row>
     <row r="14" spans="1:15" ht="90" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
+      <c r="A14" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1" t="s">
+      <c r="B14" s="7"/>
+      <c r="C14" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="D14" s="1" t="s">
+      <c r="D14" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="E14" s="1" t="s">
+      <c r="E14" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="F14" s="1" t="s">
+      <c r="F14" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="G14" s="1" t="s">
+      <c r="G14" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="H14" s="1" t="s">
+      <c r="H14" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="I14" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="J14" s="1" t="s">
+      <c r="I14" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="J14" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="K14" s="1" t="s">
+      <c r="K14" s="7" t="s">
         <v>98</v>
       </c>
       <c r="L14" s="1"/>
@@ -1380,70 +1501,70 @@
       <c r="O14" s="1"/>
     </row>
     <row r="15" spans="1:15" ht="90" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
+      <c r="A15" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1" t="s">
+      <c r="B15" s="7"/>
+      <c r="C15" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="D15" s="1" t="s">
+      <c r="D15" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="E15" s="1" t="s">
+      <c r="E15" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="F15" s="1" t="s">
+      <c r="F15" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="G15" s="1" t="s">
+      <c r="G15" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="H15" s="1" t="s">
+      <c r="H15" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="I15" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="J15" s="1" t="s">
+      <c r="I15" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="J15" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="K15" s="1"/>
+      <c r="K15" s="7"/>
       <c r="L15" s="1"/>
       <c r="M15" s="1"/>
       <c r="N15" s="1"/>
       <c r="O15" s="1"/>
     </row>
     <row r="16" spans="1:15" ht="150" x14ac:dyDescent="0.25">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="B16" s="4"/>
-      <c r="C16" s="4" t="s">
+      <c r="B16" s="8"/>
+      <c r="C16" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="D16" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="E16" s="4" t="s">
+      <c r="E16" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="F16" s="4" t="s">
+      <c r="F16" s="8" t="s">
         <v>109</v>
       </c>
-      <c r="G16" s="4" t="s">
+      <c r="G16" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="H16" s="4" t="s">
+      <c r="H16" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="I16" s="4" t="s">
+      <c r="I16" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="J16" s="4" t="s">
+      <c r="J16" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="K16" s="4" t="s">
+      <c r="K16" s="8" t="s">
         <v>108</v>
       </c>
       <c r="L16" s="4"/>
@@ -1452,136 +1573,215 @@
       <c r="O16" s="1"/>
     </row>
     <row r="17" spans="1:15" ht="75" x14ac:dyDescent="0.25">
-      <c r="A17" s="4" t="s">
+      <c r="A17" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="D17" s="4" t="s">
+      <c r="D17" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="E17" s="4" t="s">
+      <c r="E17" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="F17" s="4" t="s">
+      <c r="F17" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="G17" s="4" t="s">
+      <c r="G17" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="H17" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="I17" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="J17" s="4" t="s">
+      <c r="H17" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="I17" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J17" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="K17" s="4"/>
+      <c r="K17" s="5"/>
       <c r="L17" s="4"/>
       <c r="M17" s="1"/>
       <c r="N17" s="1"/>
       <c r="O17" s="1"/>
     </row>
     <row r="18" spans="1:15" ht="60" x14ac:dyDescent="0.25">
-      <c r="A18" s="4" t="s">
+      <c r="A18" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="B18" s="6"/>
+      <c r="C18" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="D18" s="4"/>
-      <c r="E18" s="4" t="s">
+      <c r="D18" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E18" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="F18" s="4" t="s">
+      <c r="F18" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="G18" s="4" t="s">
+      <c r="G18" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="H18" s="4" t="s">
+      <c r="H18" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="I18" s="4" t="s">
+      <c r="I18" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="J18" s="4" t="s">
+      <c r="J18" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="K18" s="4"/>
+      <c r="K18" s="5"/>
       <c r="L18" s="4"/>
       <c r="M18" s="1"/>
       <c r="N18" s="1"/>
       <c r="O18" s="1"/>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A19" s="4"/>
-      <c r="B19" s="4"/>
-      <c r="C19" s="4"/>
-      <c r="D19" s="4"/>
-      <c r="E19" s="4"/>
-      <c r="F19" s="4"/>
-      <c r="G19" s="4"/>
-      <c r="H19" s="4"/>
-      <c r="I19" s="4"/>
-      <c r="J19" s="4"/>
-      <c r="K19" s="4"/>
+    <row r="19" spans="1:15" ht="90" x14ac:dyDescent="0.25">
+      <c r="A19" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="B19" s="5"/>
+      <c r="C19" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="F19" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="G19" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H19" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="I19" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="J19" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="K19" s="5"/>
       <c r="L19" s="4"/>
       <c r="M19" s="1"/>
       <c r="N19" s="1"/>
       <c r="O19" s="1"/>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A20" s="4"/>
+    <row r="20" spans="1:15" ht="135" x14ac:dyDescent="0.25">
+      <c r="A20" s="4" t="s">
+        <v>132</v>
+      </c>
       <c r="B20" s="4"/>
-      <c r="C20" s="4"/>
-      <c r="D20" s="4"/>
-      <c r="E20" s="4"/>
-      <c r="F20" s="4"/>
-      <c r="G20" s="4"/>
-      <c r="H20" s="4"/>
-      <c r="I20" s="4"/>
-      <c r="J20" s="4"/>
-      <c r="K20" s="4"/>
+      <c r="C20" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="G20" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="H20" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="I20" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J20" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="K20" s="4" t="s">
+        <v>136</v>
+      </c>
       <c r="L20" s="4"/>
       <c r="M20" s="1"/>
       <c r="N20" s="1"/>
       <c r="O20" s="1"/>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21" s="4"/>
+    <row r="21" spans="1:15" ht="135" x14ac:dyDescent="0.25">
+      <c r="A21" s="4" t="s">
+        <v>139</v>
+      </c>
       <c r="B21" s="4"/>
-      <c r="C21" s="4"/>
-      <c r="D21" s="4"/>
-      <c r="E21" s="4"/>
-      <c r="F21" s="4"/>
-      <c r="G21" s="4"/>
-      <c r="H21" s="4"/>
-      <c r="I21" s="4"/>
-      <c r="J21" s="4"/>
-      <c r="K21" s="4"/>
+      <c r="C21" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="H21" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="I21" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J21" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="K21" s="4" t="s">
+        <v>143</v>
+      </c>
       <c r="L21" s="4"/>
       <c r="M21" s="1"/>
       <c r="N21" s="1"/>
       <c r="O21" s="1"/>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A22" s="4"/>
+    <row r="22" spans="1:15" ht="105" x14ac:dyDescent="0.25">
+      <c r="A22" s="4" t="s">
+        <v>146</v>
+      </c>
       <c r="B22" s="4"/>
-      <c r="C22" s="4"/>
-      <c r="D22" s="4"/>
-      <c r="E22" s="4"/>
-      <c r="F22" s="4"/>
-      <c r="G22" s="4"/>
-      <c r="H22" s="4"/>
-      <c r="I22" s="4"/>
-      <c r="J22" s="4"/>
+      <c r="C22" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="G22" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="H22" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="I22" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="J22" s="4" t="s">
+        <v>17</v>
+      </c>
       <c r="K22" s="4"/>
       <c r="L22" s="4"/>
     </row>

</xml_diff>

<commit_message>
agrego evidencia en video en prueba 26 interaccion rapida movil
</commit_message>
<xml_diff>
--- a/casos_de_prueba/matriz_pruebas.xlsx
+++ b/casos_de_prueba/matriz_pruebas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USUARIO\Desktop\ProyectoFinal-QA-Scarleth\casos_de_prueba\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A7745D6-785E-45A2-881C-5F6261F97351}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF916470-011A-4972-AE3A-0A03A04E53F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{5FF4DDCA-2057-4105-B76A-F7B3AA90F74B}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="185">
   <si>
     <t>ID</t>
   </si>
@@ -637,6 +637,31 @@
   </si>
   <si>
     <t xml:space="preserve">La pantalla no se fractura y adapta rapidamente a la orientacion. </t>
+  </si>
+  <si>
+    <t>CP26</t>
+  </si>
+  <si>
+    <t>Validar que el sistema maneje múltiples toques rápidos sin congelarse.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ejecutar de forma rapida. </t>
+  </si>
+  <si>
+    <t>En general funciona, pero se observó que el botón Sign up requirió doble toque en una ocasión y hubo pantallas en blanco de 1–3 s durante la carga.</t>
+  </si>
+  <si>
+    <t>1. En Safari (móvil), tocar rápidamente:
+Un pin sugerido
+Luego atras
+Luego tocar otro
+Hacerlo  3–4 veces rápido.</t>
+  </si>
+  <si>
+    <t>El sistema responde correctamente segun la rapidez de los cambios.</t>
+  </si>
+  <si>
+    <t>Evidencia en video.        PR-26_interaccion_rapida_movil.mp4</t>
   </si>
 </sst>
 </file>
@@ -2016,18 +2041,38 @@
       </c>
       <c r="L26" s="4"/>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A27" s="4"/>
+    <row r="27" spans="1:15" ht="90" x14ac:dyDescent="0.25">
+      <c r="A27" s="4" t="s">
+        <v>178</v>
+      </c>
       <c r="B27" s="4"/>
-      <c r="C27" s="4"/>
-      <c r="D27" s="4"/>
-      <c r="E27" s="4"/>
-      <c r="F27" s="4"/>
-      <c r="G27" s="4"/>
-      <c r="H27" s="4"/>
-      <c r="I27" s="4"/>
-      <c r="J27" s="4"/>
-      <c r="K27" s="4"/>
+      <c r="C27" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="G27" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="H27" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="I27" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="J27" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="K27" s="4" t="s">
+        <v>184</v>
+      </c>
       <c r="L27" s="4"/>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
agregue evidencia en video y registro de la prueba 27 responsive movil
</commit_message>
<xml_diff>
--- a/casos_de_prueba/matriz_pruebas.xlsx
+++ b/casos_de_prueba/matriz_pruebas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USUARIO\Desktop\ProyectoFinal-QA-Scarleth\casos_de_prueba\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF916470-011A-4972-AE3A-0A03A04E53F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D54E413C-DF8B-4664-BB9F-34116948CBDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{5FF4DDCA-2057-4105-B76A-F7B3AA90F74B}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="192">
   <si>
     <t>ID</t>
   </si>
@@ -71,9 +71,6 @@
     <t>Home/feed</t>
   </si>
   <si>
-    <t>1. Abrir chrome 2.Abrir pinterst. 3. Observar que sucede en los primeros segundos de la pagina.</t>
-  </si>
-  <si>
     <t>La pagina carga sin problemas.</t>
   </si>
   <si>
@@ -95,9 +92,6 @@
     <t>CP02</t>
   </si>
   <si>
-    <t xml:space="preserve"> Siempre en el home de pinterest. 1. Ir a la esquina superior izquierda a la parte de "explorar". 2. Visualizar al menos 10 imagenes de forma secuencial.</t>
-  </si>
-  <si>
     <t>Conexion estable.</t>
   </si>
   <si>
@@ -125,9 +119,6 @@
     <t xml:space="preserve">Hacer scroll continuo hasta que el sistema no cargue mas. </t>
   </si>
   <si>
-    <t xml:space="preserve">Siempre en la parte de explorar. 1. Subir y bajar continuamente. 2. Bajar la home hasta que no cargue mas. </t>
-  </si>
-  <si>
     <t>El sistema permite scroll hasta cierto límite y luego restringe contenido sin generar errores.</t>
   </si>
   <si>
@@ -149,9 +140,6 @@
     <t xml:space="preserve">Recargar la pagina estando en la parte final de la misma (donde da el limit). </t>
   </si>
   <si>
-    <t xml:space="preserve">En la parte final la pagina (cuando da el limite). 1. Presionar F5.  2. Esperar a que cargue. 3. Observar la respuesta que dio el refresh. </t>
-  </si>
-  <si>
     <t xml:space="preserve">La pagina carga nuevamente sin salirse de donde se hizo el refresh. </t>
   </si>
   <si>
@@ -168,9 +156,6 @@
   </si>
   <si>
     <t xml:space="preserve">Seleccionar 1 pin para ver la respuesta. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Tocar un pin de la feed que nos muestra. 2. Observar que aparece al clickear el pin.  </t>
   </si>
   <si>
     <t xml:space="preserve">El pin abre correctamente, mostrando la imagen seleccionada y relacionados. </t>
@@ -662,6 +647,48 @@
   </si>
   <si>
     <t>Evidencia en video.        PR-26_interaccion_rapida_movil.mp4</t>
+  </si>
+  <si>
+    <t>CP27</t>
+  </si>
+  <si>
+    <t>1. Abrir chrome                               2.Abrir pinterst.                                      3. Observar que sucede en los primeros segundos de la pagina.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Siempre en el home de pinterest.    1. Ir a la esquina superior izquierda a la parte de "explorar".                           2. Visualizar al menos 10 imagenes de forma secuencial.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Siempre en la parte de explorar.              1. Subir y bajar continuamente.            2. Bajar la home hasta que no cargue mas. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">En la parte final la pagina (cuando da el limite).                                                    1. Presionar F5.                                         2. Esperar a que cargue.                           3. Observar la respuesta que dio el refresh. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Tocar un pin de la feed que nos muestra.                                                     2. Observar que aparece al clickear el pin.  </t>
+  </si>
+  <si>
+    <t>1. En Safari iPhone, entrar a Pinterest web.
+2. Esperar a que aparezca la burbuja/mensaje de login.
+3. Intentar cerrarlo com X, “Not now” o tocar fuera 
+4. Luego intenta:
+hacer scroll
+tocar un pin sugerido (si se puede)
+tocar en la barra superior</t>
+  </si>
+  <si>
+    <t>En Safari iPhone, el login/signup aparece integrado en la página principal (como un Pin), pero aparece la burbuja al entrar a un pin sugerido. La burbuja puede cerrarse tocando fuera y permite continuar navegando sin bloqueo.</t>
+  </si>
+  <si>
+    <t>Cerrar la burburja del login y seguir navegando.</t>
+  </si>
+  <si>
+    <t>El scroll es continuo cerrando la burbuja y sin Login.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Esperar y observar lo que ocurre y cuando aparece y quitas la burbuja del Login. </t>
+  </si>
+  <si>
+    <t>Evidencia en video. PR-27_ctas_y_burbuja_login_movil.mp4</t>
   </si>
 </sst>
 </file>
@@ -1156,13 +1183,13 @@
         <v>7</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15" ht="45" x14ac:dyDescent="0.25">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
         <v>9</v>
       </c>
@@ -1170,28 +1197,28 @@
         <v>10</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E2" s="9" t="s">
+        <v>181</v>
+      </c>
+      <c r="F2" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="G2" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="9" t="s">
+      <c r="H2" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="9" t="s">
-        <v>14</v>
-      </c>
       <c r="I2" s="9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J2" s="9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K2" s="9"/>
       <c r="L2" s="1"/>
@@ -1201,32 +1228,32 @@
     </row>
     <row r="3" spans="1:15" ht="75" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B3" s="9"/>
       <c r="C3" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="F3" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="G3" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="H3" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I3" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="E3" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="F3" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="G3" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="H3" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="I3" s="9" t="s">
-        <v>24</v>
-      </c>
       <c r="J3" s="9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K3" s="9"/>
       <c r="L3" s="1"/>
@@ -1236,69 +1263,69 @@
     </row>
     <row r="4" spans="1:15" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B4" s="9"/>
       <c r="C4" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>183</v>
+      </c>
+      <c r="F4" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="G4" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="E4" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="F4" s="9" t="s">
+      <c r="H4" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I4" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="J4" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="K4" s="9" t="s">
         <v>30</v>
-      </c>
-      <c r="G4" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="H4" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="I4" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="J4" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="K4" s="9" t="s">
-        <v>33</v>
       </c>
       <c r="L4" s="1"/>
       <c r="M4" s="1"/>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
     </row>
-    <row r="5" spans="1:15" ht="75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" ht="90" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B5" s="9"/>
       <c r="C5" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>184</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="G5" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="D5" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="E5" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="F5" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="G5" s="9" t="s">
-        <v>39</v>
-      </c>
       <c r="H5" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I5" s="9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J5" s="9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K5" s="9"/>
       <c r="L5" s="1"/>
@@ -1306,34 +1333,34 @@
       <c r="N5" s="1"/>
       <c r="O5" s="1"/>
     </row>
-    <row r="6" spans="1:15" ht="75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" ht="60" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B6" s="9"/>
       <c r="C6" s="9" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>44</v>
+        <v>185</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I6" s="9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J6" s="9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K6" s="9"/>
       <c r="L6" s="1"/>
@@ -1343,32 +1370,32 @@
     </row>
     <row r="7" spans="1:15" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="B7" s="9"/>
       <c r="C7" s="9" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="G7" s="9" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="H7" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I7" s="9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J7" s="9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K7" s="9"/>
       <c r="L7" s="1"/>
@@ -1378,32 +1405,32 @@
     </row>
     <row r="8" spans="1:15" ht="105" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="B8" s="9"/>
       <c r="C8" s="9" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="E8" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="G8" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="H8" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I8" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="F8" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="G8" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="H8" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="I8" s="9" t="s">
-        <v>59</v>
-      </c>
       <c r="J8" s="9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K8" s="9"/>
       <c r="L8" s="1"/>
@@ -1413,32 +1440,32 @@
     </row>
     <row r="9" spans="1:15" ht="120" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="B9" s="9"/>
       <c r="C9" s="9" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="F9" s="9" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="G9" s="9" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="H9" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I9" s="9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J9" s="9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K9" s="9"/>
       <c r="L9" s="1"/>
@@ -1448,34 +1475,34 @@
     </row>
     <row r="10" spans="1:15" ht="75" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="F10" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="B10" s="11" t="s">
+      <c r="G10" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="C10" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="F10" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="G10" s="7" t="s">
-        <v>72</v>
-      </c>
       <c r="H10" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I10" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J10" s="7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K10" s="7"/>
       <c r="L10" s="1"/>
@@ -1485,32 +1512,32 @@
     </row>
     <row r="11" spans="1:15" ht="75" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="B11" s="7"/>
       <c r="C11" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="G11" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="H11" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="I11" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="J11" s="7" t="s">
         <v>74</v>
-      </c>
-      <c r="D11" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="E11" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="F11" s="7" t="s">
-        <v>77</v>
-      </c>
-      <c r="G11" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="H11" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="I11" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="J11" s="7" t="s">
-        <v>79</v>
       </c>
       <c r="K11" s="7"/>
       <c r="L11" s="1"/>
@@ -1520,32 +1547,32 @@
     </row>
     <row r="12" spans="1:15" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="B12" s="7"/>
       <c r="C12" s="7" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="H12" s="7" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="I12" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J12" s="7" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="K12" s="7"/>
       <c r="L12" s="1"/>
@@ -1555,32 +1582,32 @@
     </row>
     <row r="13" spans="1:15" ht="75" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="B13" s="7"/>
       <c r="C13" s="7" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I13" s="7" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J13" s="7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K13" s="7"/>
       <c r="L13" s="1"/>
@@ -1590,35 +1617,35 @@
     </row>
     <row r="14" spans="1:15" ht="90" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="B14" s="7"/>
       <c r="C14" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="G14" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="H14" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I14" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="J14" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="K14" s="7" t="s">
         <v>93</v>
-      </c>
-      <c r="D14" s="7" t="s">
-        <v>94</v>
-      </c>
-      <c r="E14" s="7" t="s">
-        <v>95</v>
-      </c>
-      <c r="F14" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="G14" s="7" t="s">
-        <v>97</v>
-      </c>
-      <c r="H14" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="I14" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="J14" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="K14" s="7" t="s">
-        <v>98</v>
       </c>
       <c r="L14" s="1"/>
       <c r="M14" s="1"/>
@@ -1627,32 +1654,32 @@
     </row>
     <row r="15" spans="1:15" ht="90" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="B15" s="7"/>
       <c r="C15" s="7" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="I15" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J15" s="7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K15" s="7"/>
       <c r="L15" s="1"/>
@@ -1662,35 +1689,35 @@
     </row>
     <row r="16" spans="1:15" ht="150" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="B16" s="8"/>
       <c r="C16" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="D16" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="D16" s="8" t="s">
-        <v>111</v>
-      </c>
       <c r="E16" s="8" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="G16" s="8" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="H16" s="8" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="I16" s="8" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J16" s="8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K16" s="8" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="L16" s="4"/>
       <c r="M16" s="1"/>
@@ -1699,34 +1726,34 @@
     </row>
     <row r="17" spans="1:15" ht="75" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="B17" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="F17" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="B17" s="12" t="s">
+      <c r="G17" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="C17" s="5" t="s">
+      <c r="H17" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I17" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="J17" s="5" t="s">
         <v>114</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>115</v>
-      </c>
-      <c r="E17" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="F17" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="G17" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="H17" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="I17" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="J17" s="5" t="s">
-        <v>119</v>
       </c>
       <c r="K17" s="5"/>
       <c r="L17" s="4"/>
@@ -1736,32 +1763,32 @@
     </row>
     <row r="18" spans="1:15" ht="60" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="B18" s="6"/>
       <c r="C18" s="5" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="I18" s="5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J18" s="5" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="K18" s="5"/>
       <c r="L18" s="4"/>
@@ -1771,32 +1798,32 @@
     </row>
     <row r="19" spans="1:15" ht="90" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="B19" s="5"/>
       <c r="C19" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="D19" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="D19" s="5" t="s">
-        <v>131</v>
-      </c>
       <c r="E19" s="5" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I19" s="5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J19" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K19" s="5"/>
       <c r="L19" s="4"/>
@@ -1806,35 +1833,35 @@
     </row>
     <row r="20" spans="1:15" ht="135" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="B20" s="5"/>
       <c r="C20" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="F20" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="G20" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="D20" s="5" t="s">
-        <v>134</v>
-      </c>
-      <c r="E20" s="5" t="s">
-        <v>135</v>
-      </c>
-      <c r="F20" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="G20" s="5" t="s">
-        <v>138</v>
-      </c>
       <c r="H20" s="5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I20" s="5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J20" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K20" s="5" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="L20" s="4"/>
       <c r="M20" s="1"/>
@@ -1843,35 +1870,35 @@
     </row>
     <row r="21" spans="1:15" ht="135" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="F21" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="G21" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="D21" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="E21" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="F21" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="G21" s="5" t="s">
-        <v>145</v>
-      </c>
       <c r="H21" s="5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I21" s="5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J21" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K21" s="5" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="L21" s="4"/>
       <c r="M21" s="1"/>
@@ -1880,213 +1907,233 @@
     </row>
     <row r="22" spans="1:15" ht="75" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="B22" s="5"/>
       <c r="C22" s="5" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I22" s="5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J22" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K22" s="5"/>
       <c r="L22" s="4"/>
     </row>
     <row r="23" spans="1:15" ht="75" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>148</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="G23" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="B23" s="13" t="s">
-        <v>153</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="D23" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="E23" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="F23" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="G23" s="4" t="s">
-        <v>157</v>
-      </c>
       <c r="H23" s="4" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="I23" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J23" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K23" s="4"/>
       <c r="L23" s="4"/>
     </row>
     <row r="24" spans="1:15" ht="135" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="G24" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="C24" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="D24" s="4" t="s">
-        <v>162</v>
-      </c>
-      <c r="E24" s="4" t="s">
-        <v>163</v>
-      </c>
-      <c r="F24" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="G24" s="4" t="s">
-        <v>164</v>
-      </c>
       <c r="H24" s="4" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="I24" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J24" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K24" s="4"/>
       <c r="L24" s="4"/>
     </row>
     <row r="25" spans="1:15" ht="105" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="H25" s="4" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="I25" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J25" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K25" s="4"/>
       <c r="L25" s="4"/>
     </row>
     <row r="26" spans="1:15" ht="75" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="B26" s="4"/>
       <c r="C26" s="4" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="E26" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="G26" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="F26" s="4" t="s">
-        <v>176</v>
-      </c>
-      <c r="G26" s="4" t="s">
-        <v>177</v>
-      </c>
       <c r="H26" s="4" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="I26" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J26" s="4" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="K26" s="4" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="L26" s="4"/>
     </row>
     <row r="27" spans="1:15" ht="90" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="G27" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="H27" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="I27" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J27" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K27" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="D27" s="4" t="s">
+      <c r="L27" s="4"/>
+    </row>
+    <row r="28" spans="1:15" ht="165" x14ac:dyDescent="0.25">
+      <c r="A28" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="E27" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="F27" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="G27" s="4" t="s">
-        <v>181</v>
-      </c>
-      <c r="H27" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="I27" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="J27" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="K27" s="4" t="s">
-        <v>184</v>
-      </c>
-      <c r="L27" s="4"/>
-    </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A28" s="4"/>
       <c r="B28" s="4"/>
-      <c r="C28" s="4"/>
-      <c r="D28" s="4"/>
-      <c r="E28" s="4"/>
-      <c r="F28" s="4"/>
-      <c r="G28" s="4"/>
-      <c r="H28" s="4"/>
-      <c r="I28" s="4"/>
-      <c r="J28" s="4"/>
-      <c r="K28" s="4"/>
+      <c r="C28" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="F28" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="G28" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="H28" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="I28" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="J28" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="K28" s="4" t="s">
+        <v>191</v>
+      </c>
       <c r="L28" s="4"/>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
agrego evidencias de prueba 28 teclado y sugerencias de busqueda
</commit_message>
<xml_diff>
--- a/casos_de_prueba/matriz_pruebas.xlsx
+++ b/casos_de_prueba/matriz_pruebas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USUARIO\Desktop\ProyectoFinal-QA-Scarleth\casos_de_prueba\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D54E413C-DF8B-4664-BB9F-34116948CBDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11F3458A-6216-4F4B-9973-E7C467C8D79F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{5FF4DDCA-2057-4105-B76A-F7B3AA90F74B}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="199">
   <si>
     <t>ID</t>
   </si>
@@ -689,6 +689,34 @@
   </si>
   <si>
     <t>Evidencia en video. PR-27_ctas_y_burbuja_login_movil.mp4</t>
+  </si>
+  <si>
+    <t>CP28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validar los cambios en la feel al activar el teclado del movil. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buscar la barra de buscar para ejecutar la prueba. </t>
+  </si>
+  <si>
+    <t>1. En el movil (safari) abrir el teclado:
+-Abrir Pinterest web.
+-Tocar la barra de búsqueda (si aparece). Si no aparece en home, abrir un pin primero y luego tocar búsqueda.
+-Espera a que aparezca el teclado.                                                       2. Tocar “cerrar"  o fuera del campo.
+Observar si:
+-El teclado desaparece correctamente.
+-El layout vuelve a su posición original.
+-No quedan espacios vacíos extraños.</t>
+  </si>
+  <si>
+    <t>El teclado no provoca ningun cambio funcional del sistema.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El teclado se activo y cerro de forma normal. </t>
+  </si>
+  <si>
+    <t>El teclado no mostro ningun error al ser activado; sin embargo, al borrar el filtro (palabra) que estaba por default del pin abierto, no mostraba resultados de imagenes mas que de filtro sugeridos.              PR-28_teclado_sugerencias_pin.png,                        PR-28_busqueda_vacia_mantiene_sugerencias.png</t>
   </si>
 </sst>
 </file>
@@ -729,7 +757,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -754,6 +782,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFE1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -767,7 +801,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -803,15 +837,24 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFFFFE1"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1938,258 +1981,279 @@
       <c r="L22" s="4"/>
     </row>
     <row r="23" spans="1:15" ht="75" x14ac:dyDescent="0.25">
-      <c r="A23" s="4" t="s">
+      <c r="A23" s="13" t="s">
         <v>147</v>
       </c>
-      <c r="B23" s="13" t="s">
+      <c r="B23" s="14" t="s">
         <v>148</v>
       </c>
-      <c r="C23" s="4" t="s">
+      <c r="C23" s="13" t="s">
         <v>149</v>
       </c>
-      <c r="D23" s="4" t="s">
+      <c r="D23" s="13" t="s">
         <v>150</v>
       </c>
-      <c r="E23" s="4" t="s">
+      <c r="E23" s="13" t="s">
         <v>153</v>
       </c>
-      <c r="F23" s="4" t="s">
+      <c r="F23" s="13" t="s">
         <v>151</v>
       </c>
-      <c r="G23" s="4" t="s">
+      <c r="G23" s="13" t="s">
         <v>152</v>
       </c>
-      <c r="H23" s="4" t="s">
+      <c r="H23" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="I23" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="J23" s="4" t="s">
+      <c r="I23" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="J23" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="K23" s="4"/>
+      <c r="K23" s="13"/>
       <c r="L23" s="4"/>
     </row>
     <row r="24" spans="1:15" ht="135" x14ac:dyDescent="0.25">
-      <c r="A24" s="4" t="s">
+      <c r="A24" s="13" t="s">
         <v>154</v>
       </c>
-      <c r="C24" s="4" t="s">
+      <c r="B24" s="15"/>
+      <c r="C24" s="13" t="s">
         <v>155</v>
       </c>
-      <c r="D24" s="4" t="s">
+      <c r="D24" s="13" t="s">
         <v>157</v>
       </c>
-      <c r="E24" s="4" t="s">
+      <c r="E24" s="13" t="s">
         <v>158</v>
       </c>
-      <c r="F24" s="4" t="s">
+      <c r="F24" s="13" t="s">
         <v>156</v>
       </c>
-      <c r="G24" s="4" t="s">
+      <c r="G24" s="13" t="s">
         <v>159</v>
       </c>
-      <c r="H24" s="4" t="s">
+      <c r="H24" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="I24" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="J24" s="4" t="s">
+      <c r="I24" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="J24" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="K24" s="4"/>
+      <c r="K24" s="13"/>
       <c r="L24" s="4"/>
     </row>
     <row r="25" spans="1:15" ht="105" x14ac:dyDescent="0.25">
-      <c r="A25" s="4" t="s">
+      <c r="A25" s="13" t="s">
         <v>160</v>
       </c>
-      <c r="B25" s="4"/>
-      <c r="C25" s="4" t="s">
+      <c r="B25" s="13"/>
+      <c r="C25" s="13" t="s">
         <v>161</v>
       </c>
-      <c r="D25" s="4" t="s">
+      <c r="D25" s="13" t="s">
         <v>162</v>
       </c>
-      <c r="E25" s="4" t="s">
+      <c r="E25" s="13" t="s">
         <v>163</v>
       </c>
-      <c r="F25" s="4" t="s">
+      <c r="F25" s="13" t="s">
         <v>164</v>
       </c>
-      <c r="G25" s="4" t="s">
+      <c r="G25" s="13" t="s">
         <v>165</v>
       </c>
-      <c r="H25" s="4" t="s">
+      <c r="H25" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="I25" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="J25" s="4" t="s">
+      <c r="I25" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="J25" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="K25" s="4"/>
+      <c r="K25" s="13"/>
       <c r="L25" s="4"/>
     </row>
     <row r="26" spans="1:15" ht="75" x14ac:dyDescent="0.25">
-      <c r="A26" s="4" t="s">
+      <c r="A26" s="13" t="s">
         <v>166</v>
       </c>
-      <c r="B26" s="4"/>
-      <c r="C26" s="4" t="s">
+      <c r="B26" s="13"/>
+      <c r="C26" s="13" t="s">
         <v>168</v>
       </c>
-      <c r="D26" s="4" t="s">
+      <c r="D26" s="13" t="s">
         <v>169</v>
       </c>
-      <c r="E26" s="4" t="s">
+      <c r="E26" s="13" t="s">
         <v>167</v>
       </c>
-      <c r="F26" s="4" t="s">
+      <c r="F26" s="13" t="s">
         <v>171</v>
       </c>
-      <c r="G26" s="4" t="s">
+      <c r="G26" s="13" t="s">
         <v>172</v>
       </c>
-      <c r="H26" s="4" t="s">
+      <c r="H26" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="I26" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="J26" s="4" t="s">
+      <c r="I26" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="J26" s="13" t="s">
         <v>114</v>
       </c>
-      <c r="K26" s="4" t="s">
+      <c r="K26" s="13" t="s">
         <v>170</v>
       </c>
       <c r="L26" s="4"/>
     </row>
     <row r="27" spans="1:15" ht="90" x14ac:dyDescent="0.25">
-      <c r="A27" s="4" t="s">
+      <c r="A27" s="13" t="s">
         <v>173</v>
       </c>
-      <c r="B27" s="4"/>
-      <c r="C27" s="4" t="s">
+      <c r="B27" s="13"/>
+      <c r="C27" s="13" t="s">
         <v>174</v>
       </c>
-      <c r="D27" s="4" t="s">
+      <c r="D27" s="13" t="s">
         <v>175</v>
       </c>
-      <c r="E27" s="4" t="s">
+      <c r="E27" s="13" t="s">
         <v>177</v>
       </c>
-      <c r="F27" s="4" t="s">
+      <c r="F27" s="13" t="s">
         <v>178</v>
       </c>
-      <c r="G27" s="4" t="s">
+      <c r="G27" s="13" t="s">
         <v>176</v>
       </c>
-      <c r="H27" s="4" t="s">
+      <c r="H27" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="I27" s="4" t="s">
+      <c r="I27" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="J27" s="4" t="s">
+      <c r="J27" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="K27" s="4" t="s">
+      <c r="K27" s="13" t="s">
         <v>179</v>
       </c>
       <c r="L27" s="4"/>
     </row>
     <row r="28" spans="1:15" ht="165" x14ac:dyDescent="0.25">
-      <c r="A28" s="4" t="s">
+      <c r="A28" s="13" t="s">
         <v>180</v>
       </c>
-      <c r="B28" s="4"/>
-      <c r="C28" s="4" t="s">
+      <c r="B28" s="13"/>
+      <c r="C28" s="13" t="s">
         <v>188</v>
       </c>
-      <c r="D28" s="4" t="s">
+      <c r="D28" s="13" t="s">
         <v>190</v>
       </c>
-      <c r="E28" s="4" t="s">
+      <c r="E28" s="13" t="s">
         <v>186</v>
       </c>
-      <c r="F28" s="4" t="s">
+      <c r="F28" s="13" t="s">
         <v>189</v>
       </c>
-      <c r="G28" s="4" t="s">
+      <c r="G28" s="13" t="s">
         <v>187</v>
       </c>
-      <c r="H28" s="4" t="s">
+      <c r="H28" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="I28" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="J28" s="4" t="s">
+      <c r="I28" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="J28" s="13" t="s">
         <v>114</v>
       </c>
-      <c r="K28" s="4" t="s">
+      <c r="K28" s="13" t="s">
         <v>191</v>
       </c>
       <c r="L28" s="4"/>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A29" s="4"/>
-      <c r="B29" s="4"/>
-      <c r="C29" s="4"/>
-      <c r="D29" s="4"/>
-      <c r="E29" s="4"/>
-      <c r="F29" s="4"/>
-      <c r="G29" s="4"/>
-      <c r="H29" s="4"/>
-      <c r="I29" s="4"/>
-      <c r="J29" s="4"/>
-      <c r="K29" s="4"/>
+    <row r="29" spans="1:15" ht="270" x14ac:dyDescent="0.25">
+      <c r="A29" s="13" t="s">
+        <v>192</v>
+      </c>
+      <c r="B29" s="13"/>
+      <c r="C29" s="13" t="s">
+        <v>193</v>
+      </c>
+      <c r="D29" s="13" t="s">
+        <v>194</v>
+      </c>
+      <c r="E29" s="13" t="s">
+        <v>195</v>
+      </c>
+      <c r="F29" s="13" t="s">
+        <v>196</v>
+      </c>
+      <c r="G29" s="13" t="s">
+        <v>197</v>
+      </c>
+      <c r="H29" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="I29" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="J29" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="K29" s="13" t="s">
+        <v>198</v>
+      </c>
       <c r="L29" s="4"/>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A30" s="4"/>
-      <c r="B30" s="4"/>
-      <c r="C30" s="4"/>
-      <c r="D30" s="4"/>
-      <c r="E30" s="4"/>
-      <c r="F30" s="4"/>
-      <c r="G30" s="4"/>
-      <c r="H30" s="4"/>
-      <c r="I30" s="4"/>
-      <c r="J30" s="4"/>
-      <c r="K30" s="4"/>
+      <c r="A30" s="13"/>
+      <c r="B30" s="13"/>
+      <c r="C30" s="13"/>
+      <c r="D30" s="13"/>
+      <c r="E30" s="13"/>
+      <c r="F30" s="13"/>
+      <c r="G30" s="13"/>
+      <c r="H30" s="13"/>
+      <c r="I30" s="13"/>
+      <c r="J30" s="13"/>
+      <c r="K30" s="13"/>
       <c r="L30" s="4"/>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A31" s="4"/>
-      <c r="B31" s="4"/>
-      <c r="C31" s="4"/>
-      <c r="D31" s="4"/>
-      <c r="E31" s="4"/>
-      <c r="F31" s="4"/>
-      <c r="G31" s="4"/>
-      <c r="H31" s="4"/>
-      <c r="I31" s="4"/>
-      <c r="J31" s="4"/>
-      <c r="K31" s="4"/>
+      <c r="A31" s="13"/>
+      <c r="B31" s="13"/>
+      <c r="C31" s="13"/>
+      <c r="D31" s="13"/>
+      <c r="E31" s="13"/>
+      <c r="F31" s="13"/>
+      <c r="G31" s="13"/>
+      <c r="H31" s="13"/>
+      <c r="I31" s="13"/>
+      <c r="J31" s="13"/>
+      <c r="K31" s="13"/>
       <c r="L31" s="4"/>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A32" s="4"/>
-      <c r="B32" s="4"/>
-      <c r="C32" s="4"/>
-      <c r="D32" s="4"/>
-      <c r="E32" s="4"/>
-      <c r="F32" s="4"/>
-      <c r="G32" s="4"/>
-      <c r="H32" s="4"/>
-      <c r="I32" s="4"/>
-      <c r="J32" s="4"/>
-      <c r="K32" s="4"/>
+      <c r="A32" s="13"/>
+      <c r="B32" s="13"/>
+      <c r="C32" s="13"/>
+      <c r="D32" s="13"/>
+      <c r="E32" s="13"/>
+      <c r="F32" s="13"/>
+      <c r="G32" s="13"/>
+      <c r="H32" s="13"/>
+      <c r="I32" s="13"/>
+      <c r="J32" s="13"/>
+      <c r="K32" s="13"/>
       <c r="L32" s="4"/>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
agregue evidencias en video y screenshot de prueba 30 modo offline y recuperacion
</commit_message>
<xml_diff>
--- a/casos_de_prueba/matriz_pruebas.xlsx
+++ b/casos_de_prueba/matriz_pruebas.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USUARIO\Desktop\ProyectoFinal-QA-Scarleth\casos_de_prueba\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11F3458A-6216-4F4B-9973-E7C467C8D79F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E592C73-5E90-450B-8324-12AF9A7AD689}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{5FF4DDCA-2057-4105-B76A-F7B3AA90F74B}"/>
   </bookViews>
   <sheets>
-    <sheet name="Casos-de-prueba" sheetId="1" r:id="rId1"/>
+    <sheet name="Casos-de-prueba-pinterest" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="212">
   <si>
     <t>ID</t>
   </si>
@@ -655,9 +655,6 @@
     <t>1. Abrir chrome                               2.Abrir pinterst.                                      3. Observar que sucede en los primeros segundos de la pagina.</t>
   </si>
   <si>
-    <t xml:space="preserve"> Siempre en el home de pinterest.    1. Ir a la esquina superior izquierda a la parte de "explorar".                           2. Visualizar al menos 10 imagenes de forma secuencial.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Siempre en la parte de explorar.              1. Subir y bajar continuamente.            2. Bajar la home hasta que no cargue mas. </t>
   </si>
   <si>
@@ -716,7 +713,55 @@
     <t xml:space="preserve">El teclado se activo y cerro de forma normal. </t>
   </si>
   <si>
-    <t>El teclado no mostro ningun error al ser activado; sin embargo, al borrar el filtro (palabra) que estaba por default del pin abierto, no mostraba resultados de imagenes mas que de filtro sugeridos.              PR-28_teclado_sugerencias_pin.png,                        PR-28_busqueda_vacia_mantiene_sugerencias.png</t>
+    <t>El teclado no mostro ningun error al ser activado; sin embargo, al borrar el filtro (palabra) que estaba por default del pin abierto, no mostraba resultados de imagenes mas que de filtro sugeridos.              PR-28_teclado_sugerencias_pin.jpeg,                        PR-28_busqueda_vacia_mantiene_sugerencias.jpeg</t>
+  </si>
+  <si>
+    <t>CP29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validar la fluidez de respuesta del boton de atras. </t>
+  </si>
+  <si>
+    <t>Tocar el boton de atras varias veces.</t>
+  </si>
+  <si>
+    <t>Siempre desde pinterest del movil (safari)                                                       1. Abrir Pinterest web.
+2. Abrir un pin.
+3. Desde ese pin abrir otro pin sugerido.                                                    4 Luego tocar el botón Atrás del navegador.
+5. Repetir Atrás 2–3 veces.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La feed sigue funcionando con estabilidad despues de varios retrocesos. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">El boton de atras tiene resultados estables, sin perder el pin principal o dejar espacios en blanco al hacerlo rapido. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">CP30 </t>
+  </si>
+  <si>
+    <t>Verificar cómo responde el sitio si la conexión cambia momentáneamente.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Siempre en el home de pinterest.    1. Ir a la esquina superior izquierda a la parte de "explorar".                       2. Visualizar al menos 10 imagenes de forma secuencial.</t>
+  </si>
+  <si>
+    <t>Realizar ejecucion tipo Stress.</t>
+  </si>
+  <si>
+    <t>1.Abrir Pinterest en Safari.
+2. Mientras está cargando contenido (haciendo scroll), desactivar el wifin por 3–4 segundos.
+3. Hacer scroll varias veces, regresar, siguiente, regresar.           4. Activar nuavemente el wifi.
+5. Observar qué ocurre.</t>
+  </si>
+  <si>
+    <t>Al desactivar Wi-Fi el sistema muestra mensaje de sin conexión y algunos pines quedan sin cargar. Al reactivar Wi-Fi, el sistema se recupera automáticamente y continúa cargando contenido sin requerir refresh manual.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La pagina no borra las busquedas o elementos cargados al desactivar el wifi. </t>
+  </si>
+  <si>
+    <t>Evidencia en tipo video y screenshot:                   PR-30_modo_offline_recuperacion_automatica.mp4,                                    PR-30_mensaje_sin_conexion.jpeg,                          PR-30_pin_no_carga_offline.jpeg</t>
   </si>
 </sst>
 </file>
@@ -801,7 +846,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -844,6 +889,9 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1281,7 +1329,7 @@
         <v>20</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>182</v>
+        <v>206</v>
       </c>
       <c r="F3" s="9" t="s">
         <v>21</v>
@@ -1315,8 +1363,8 @@
       <c r="D4" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="E4" s="9" t="s">
-        <v>183</v>
+      <c r="E4" s="16" t="s">
+        <v>182</v>
       </c>
       <c r="F4" s="9" t="s">
         <v>27</v>
@@ -1353,7 +1401,7 @@
         <v>33</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="F5" s="9" t="s">
         <v>34</v>
@@ -1388,7 +1436,7 @@
         <v>39</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F6" s="9" t="s">
         <v>40</v>
@@ -2152,19 +2200,19 @@
       </c>
       <c r="B28" s="13"/>
       <c r="C28" s="13" t="s">
+        <v>187</v>
+      </c>
+      <c r="D28" s="13" t="s">
+        <v>189</v>
+      </c>
+      <c r="E28" s="13" t="s">
+        <v>185</v>
+      </c>
+      <c r="F28" s="13" t="s">
         <v>188</v>
       </c>
-      <c r="D28" s="13" t="s">
-        <v>190</v>
-      </c>
-      <c r="E28" s="13" t="s">
+      <c r="G28" s="13" t="s">
         <v>186</v>
-      </c>
-      <c r="F28" s="13" t="s">
-        <v>189</v>
-      </c>
-      <c r="G28" s="13" t="s">
-        <v>187</v>
       </c>
       <c r="H28" s="13" t="s">
         <v>22</v>
@@ -2176,29 +2224,29 @@
         <v>114</v>
       </c>
       <c r="K28" s="13" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="L28" s="4"/>
     </row>
     <row r="29" spans="1:15" ht="270" x14ac:dyDescent="0.25">
       <c r="A29" s="13" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B29" s="13"/>
       <c r="C29" s="13" t="s">
+        <v>192</v>
+      </c>
+      <c r="D29" s="13" t="s">
         <v>193</v>
       </c>
-      <c r="D29" s="13" t="s">
+      <c r="E29" s="13" t="s">
         <v>194</v>
       </c>
-      <c r="E29" s="13" t="s">
+      <c r="F29" s="13" t="s">
         <v>195</v>
       </c>
-      <c r="F29" s="13" t="s">
+      <c r="G29" s="13" t="s">
         <v>196</v>
-      </c>
-      <c r="G29" s="13" t="s">
-        <v>197</v>
       </c>
       <c r="H29" s="13" t="s">
         <v>14</v>
@@ -2210,36 +2258,74 @@
         <v>16</v>
       </c>
       <c r="K29" s="13" t="s">
+        <v>197</v>
+      </c>
+      <c r="L29" s="4"/>
+    </row>
+    <row r="30" spans="1:15" ht="135" x14ac:dyDescent="0.25">
+      <c r="A30" s="13" t="s">
         <v>198</v>
       </c>
-      <c r="L29" s="4"/>
-    </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A30" s="13"/>
       <c r="B30" s="13"/>
-      <c r="C30" s="13"/>
-      <c r="D30" s="13"/>
-      <c r="E30" s="13"/>
-      <c r="F30" s="13"/>
-      <c r="G30" s="13"/>
-      <c r="H30" s="13"/>
-      <c r="I30" s="13"/>
-      <c r="J30" s="13"/>
+      <c r="C30" s="13" t="s">
+        <v>199</v>
+      </c>
+      <c r="D30" s="13" t="s">
+        <v>200</v>
+      </c>
+      <c r="E30" s="13" t="s">
+        <v>201</v>
+      </c>
+      <c r="F30" s="13" t="s">
+        <v>202</v>
+      </c>
+      <c r="G30" s="13" t="s">
+        <v>203</v>
+      </c>
+      <c r="H30" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="I30" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="J30" s="13" t="s">
+        <v>16</v>
+      </c>
       <c r="K30" s="13"/>
       <c r="L30" s="4"/>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A31" s="13"/>
+    <row r="31" spans="1:15" ht="180" x14ac:dyDescent="0.25">
+      <c r="A31" s="13" t="s">
+        <v>204</v>
+      </c>
       <c r="B31" s="13"/>
-      <c r="C31" s="13"/>
-      <c r="D31" s="13"/>
-      <c r="E31" s="13"/>
-      <c r="F31" s="13"/>
-      <c r="G31" s="13"/>
-      <c r="H31" s="13"/>
-      <c r="I31" s="13"/>
-      <c r="J31" s="13"/>
-      <c r="K31" s="13"/>
+      <c r="C31" s="13" t="s">
+        <v>205</v>
+      </c>
+      <c r="D31" s="13" t="s">
+        <v>207</v>
+      </c>
+      <c r="E31" s="13" t="s">
+        <v>208</v>
+      </c>
+      <c r="F31" s="13" t="s">
+        <v>210</v>
+      </c>
+      <c r="G31" s="13" t="s">
+        <v>209</v>
+      </c>
+      <c r="H31" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="I31" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="J31" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="K31" s="13" t="s">
+        <v>211</v>
+      </c>
       <c r="L31" s="4"/>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.25">

</xml_diff>